<commit_message>
Correct the metadata on the agent emplate and update hash
</commit_message>
<xml_diff>
--- a/public/Bulk_Securities_Transfer_Charge_template_v1a.xlsx
+++ b/public/Bulk_Securities_Transfer_Charge_template_v1a.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tapiwa/Desktop/stf templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jhumble/work/securities-transfer-charge-frontend/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D608453-E419-6242-939B-8A824F0C0D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4AB7DD-87A7-A24F-B857-1A50257DA9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="44160" windowHeight="24880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -796,13 +796,13 @@
         <v>70</v>
       </c>
       <c r="X1" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Y1" s="11" t="s">
         <v>72</v>
       </c>
       <c r="Z1" s="11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="AA1" s="11" t="s">
         <v>76</v>
@@ -1249,7 +1249,6 @@
       <c r="U8" s="8"/>
       <c r="V8" s="8"/>
       <c r="W8" s="8"/>
-      <c r="X8" s="8"/>
       <c r="Y8" s="8"/>
       <c r="Z8" s="8"/>
       <c r="AA8" s="8"/>

</xml_diff>